<commit_message>
Update debates data - 2026-03-04
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -132,6 +132,208 @@
   </si>
   <si>
     <t xml:space="preserve">Ich sage es gleich vorweg: Dieser Antrag zur Regionalpolitik bereitet mir keine Freude. Wenn ich meinen Kanton Bern vertreten möchte, müsste ich klar gegen diese Kürzung stimmen, denn er profitiert erheblich von der Finanzierung der NRP-Projekte. Das mache ich aber nicht, weil es beim EP 27 nicht um einzelne Parlamentarier, einzelne Kantone oder Partikularinteressen geht. Es geht darum, die Gesamtinteressen des Bundeshaushaltes und die Einhaltung der bewährten Schuldenbremse im Blick zu behalten. Wenn jeder sein eigenes "Gärtli" verteidigt, kommen wir auf keinen grünen Zweig. Es bleibt dabei: Man kann das Fell des Bären nicht waschen, ohne es nass zu machen. Das übergeordnete Ziel ist es, eine Lösung zu finden, um das strukturelle Defizit in den Griff zu bekommen. Hier geht es nicht um eine eigentliche Sparmassnahme in der Regionalpolitik, sondern darum, einen Fonds auf ein angemessenes Niveau zu bringen. Sein Eigenkapital beträgt eine Milliarde Franken, seine Liquidität rund eine halbe Milliarde Franken. Selbst die Eidgenössische Finanzkontrolle hat kürzlich kritisiert, dass der Fonds massiv überdotiert ist. Es geht darum, in den nächsten drei Jahren 50 Millionen Franken einzusparen, also 5 Prozent. Für mich ist entscheidend, ob ein reifes Regionalprojekt nicht realisiert werden kann. Die Verwaltung hat diese Frage klar verneint. Dementsprechend kann man hier den Bundesrat und damit meine Minderheit bedenkenlos unterstützen. Die Regionalpolitik wird dadurch in keiner Weise geschwächt. Die vorübergehende Kürzung ist gut verkraftbar. Besten Dank, wenn Sie mich dabei unterstützen.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">369707</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260304</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Page Pierre-André</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ziff. 34
+Antrag der Mehrheit [GZ]
+Art. 10b Titel [GZ]
+Zusammenarbeit des EFD, der FINMA und der Nationalbank zur Abwendung und Bewältigung des Ausfalls einer systemrelevanten Bank
+Art. 10b Text [GZ]
+Schätzt die FINMA, insbesondere nach Beurteilung der Risiken bei einer systemrelevanten Bank, die Anordnung einer Massnahme nach Artikel 25 Absatz 1 als voraussichtlich notwendig ein, teilt sie ihre Einschätzung unverzüglich dem EFD und der Nationalbank mit. Nach Benachrichtigung durch die FINMA teil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ziff. 34
+Antrag der Mehrheit [GZ]
+Art. 10b Titel [GZ]
+Zusammenarbeit des EFD, der FINMA und der Nationalbank zur Abwendung und Bewältigung des Ausfalls einer systemrelevanten Bank
+Art. 10b Text [GZ]
+Schätzt die FINMA, insbesondere nach Beurteilung der Risiken bei einer systemrelevanten Bank, die Anordnung einer Massnahme nach Artikel 25 Absatz 1 als voraussichtlich notwendig ein, teilt sie ihre Einschätzung unverzüglich dem EFD und der Nationalbank mit. Nach Benachrichtigung durch die FINMA teilt die Nationalbank dem EFD ihre Einschätzung insbesondere in Bezug auf die Risiken für die Schweizer Volkswirtschaft und das schweizerische Finanzsystem mit.
+Art. 30b Abs. 3 Bst. a[GZ]
+a. privilegierte Forderungen der ersten und zweiten Klasse nach Artikel 219 Absatz 4 SchKG sowie Forderungen nach Artikel 32c Absatz 1: im Umfang ihrer Privilegierung;
+Elfter a. Abschnitt Titel[GZ]
+Gewährung von Ausfallgarantien des Bundes für Liquiditätshilfe-Darlehen der Nationalbank an systemrelevante Banken
+Art. 32a Titel [GZ]
+Ausfallgarantien
+Art. 32a Abs. 1 [GZ]
+Der Bund kann der Nationalbank subsidiäre Ausfallgarantien gewähren für Liquiditätshilfe-Darlehen an Banken, die systemrelevant oder Teil einer systemrelevanten Finanzgruppe sind, sofern:
+a. das Verfahren zur Sanierung der Darlehensnehmerin eingeleitet worden ist oder dessen Einleitung bevorsteht; und
+b. ohne Gewährung solcher Darlehen eine erhebliche Schädigung der Schweizer Volkswirtschaft und des schweizerischen Finanzsystems droht.
+Art. 32a Abs. 2 [GZ]
+Der Bund erhebt von den Banken, die systemrelevant oder Teil einer systemrelevanten Finanzgruppe sind, jährlich eine Pauschale für das Risiko einer allfälligen Bereitstellung einer Ausfallgarantie. Die Pauschale entspricht dem Produkt aus einem einheitlichen Bemessungssatz und einer für jede Bank berechneten Bemessungsgrundlage. 
+Art. 32a Abs. 3 [GZ]
+Der Bund hat Anspruch auf eine Prämie für die Bereitstellung einer Ausfallgarantie. Die Bereitstellungsprämie bemisst sich nach der Höhe der Ausfallgarantie. 
+32a Abs. 4 [GZ]
+Der Bund und die Nationalbank haben Anspruch auf je eine Risikoprämie zur Abgeltung der mit einem Liquiditätshilfe-Darlehen mit Ausfallgarantie übernommenen Risiken. Die Risikoprämien bemessen sich nach der Höhe der ausbezahlten Liquiditätshilfe-Darlehen mit Ausfallgarantie. 
+Art. 32a Abs. 5 [GZ]
+Die Nationalbank hat Anspruch auf Zinsen auf Liquiditätshilfe-Darlehen mit Ausfallgarantie.
+Art. 32a Abs. 6 [GZ]
+Kosten für Leistungen Dritter, die im Zusammenhang mit Liquiditätshilfe-Darlehen mit Ausfallgarantie beim Bund, der Nationalbank oder der FINMA entstehen, werden der Darlehensnehmerin auferlegt.
+Art. 32a Abs. 7 [GZ]
+Der Bundesrat regelt namentlich:
+a. welche Massnahmen die Darlehensnehmerin ausgeschöpft haben muss, um sich Finanzierungsquellen zu erschliessen oder Sicherheiten zu beschaffen;
+b. den Bemessungssatz und die Berechnungsgrundlage der Pauschale sowie die Bemessung und Berechnung der Bereitstellungsprämie, der Risikoprämien und der Zinsen und deren jeweilige Erhebung;
+c. wann und in welchem Umfang der Anspruch der Nationalbank auf Übernahme eines definitiven Verlusts aus den von ihr gewährten Liquiditätshilfe-Darlehen mit Ausfallgarantie entsteht und unter welchen Voraussetzungen fällig wird;
+d. die weiteren Voraussetzungen zur Inanspruchnahme von Liquiditätshilfe-Darlehens mit Ausfallgarantie, namentlich notwendige Bestätigungen der FINMA und der Nationalbank;
+e. die Pflichten der FINMA und der Nationalbank im Zusammenhang mit der Risikoreduktion, Überwachung und Berichterstattung.
+Art. 32b Titel [GZ]
+Pflichten der Darlehensnehmerin als Folge von Liquiditätshilfe-Darlehen mit Ausfallgarantie
+Art. 32b Abs. 1 [GZ]
+Der Darlehensnehmerin und ihren direkten oder indirekten Tochtergesellschaften sind nicht erlaubt:
+a. die Beschlussfassung über und die Auszahlung von Dividenden und Tantiemen an Personen inner- und ausserhalb des Konzerns der Darlehensnehmerin
+b. die Rückerstattung von hartem Kernkapital, zusätzlichem Kernkapital, Ergänzungskapital und zusätzlichen verlustabsorbierenden Mitteln;
+c. die Gewährung von Darlehen an die und die Rückzahlung von Darlehen der Eigentümer der Konzernobergesellschaft.
+Art. 32b Abs. 2 [GZ]
+Die Darlehensnehmerin und die mit ihr direkt oder indirekt verbundenen Konzerngesellschaften dürfen weder Handlungen vornehmen, die die Rückzahlung der Liquiditätshilfe-Darlehen mit Ausfallgarantie und die vollständige Begleichung der Zinsen und Prämien nach Artikel 32a verzögern oder gefährden könnten, noch dürfen sie Handlungen unterlassen, die der Rückzahlung dieser Darlehen und der vollständigen Begleichung dieser Zinsen und Prämien dienlich sind. 
+Art. 32b Abs. 3 [GZ]
+Die Darlehensnehmerin muss die Liquiditätshilfe-Darlehen mit Ausfallgarantie vor anderen Liquiditätshilfe-Darlehen, die die Nationalbank ihr gewährt hat, zurückzahlen.
+Art. 32b Abs. 4 [GZ]
+Der Bundesrat regelt die Pflichten der Darlehensnehmerin einschliesslich der Ausnahmen:
+a. von den Pflichten der Darlehensnehmerin nach den Absätzen 1 und 2, insbesondere für die Fälle:
+1. vorbestehender ordentlicher Zahlungspflichten in Bezug auf Zinsen oder Amortisationen in Zusammenhang mit Geschäften nach Absatz 1 Buchstaben b oder c; und
+2. wenn die Darlehensnehmerin oder die Finanzgruppe von einer Drittgesellschaft übernommen und die Darlehensnehmerin oder die Finanzgruppe von einer Einheit der Drittgesellschaft absorbiert wird.
+b. von der Pflicht zur vorrangigen Rückzahlung der Liquiditätshilfe-Darlehen mit Ausfallgarantie.
+Art. 32c Titel [GZ]
+Konkursprivileg für Forderungen aus Liquiditätshilfe-Darlehen mit Ausfallgarantie
+Art. 32c Abs. 1 [GZ]
+Forderungen der Nationalbank aus Liquiditätshilfe-Darlehen mit Ausfallgarantie, die aufgelaufenen Prämien der Nationalbank und des Bundes und die aufgelaufenen Zinsen werden der dritten Klasse nach Artikel 219 Absatz 4 SchKG zugewiesen. 
+Art. 32c Abs. 2 [GZ]
+Sofern solche Forderungen bestehen, sind in Abweichung von Artikel 220 Absatz 1 SchKG die Forderungen innerhalb der dritten Klasse nach folgender Rangordnung zu befriedigen:
+a. Forderungen aus Freizügigkeitskonten in Form der reinen Sparlösung, die vom Bundesrat gestützt auf Artikel 26 Absatz 1 des Freizügigkeitsgesetzes vom 17. Dezember 1993 vorgesehen werden, und Forderungen aus Spareinlagen auf Konten der gebundenen Selbstvorsorge nach Artikel 82 Absatz 1 Buchstabe b des Bundesgesetzes vom 25. Juni 1982 über die berufliche Alters-, Hinterlassenen- und Invalidenvorsorge; 
+b. Forderungen der Nationalbank aus Liquiditätshilfe-Darlehen mit Ausfallgarantie, die aufgelaufenen Prämien der Nationalbank und des Bundes und die aufgelaufenen Zinsen; 
+c. alle übrigen Forderungen der dritten Klasse.
+Art. 32d Titel [GZ]
+Datenbearbeitung und Informationsaustausch 
+Art. 32d Abs. 1 [GZ]
+Das EFD, die FINMA, die Nationalbank und die Eidgenössische Finanzkontrolle sowie die für den Vollzug dieses Abschnitts beigezogenen Dritten dürfen Personendaten und Daten juristischer Personen, einschliesslich besonders schützenswerter Daten nach Artikel 5 Buchstabe c Ziffern 1, 2, 5 und 6 des Datenschutzgesetzes vom 25. September 2020 und besonders schützenswerter Daten juristischer Personen nach Artikel 57r Absatz 2 des Regierungs- und Verwaltungsorganisationsgesetzes vom 21. März 1997, und andere Informationen bearbeiten und einander bekanntgeben, soweit dies für den Vollzug dieses Abschnitts, namentlich für die Gewährung, Verwaltung, Überwachung, Prüfung und Abwicklung von Liquiditätshilfe-Darlehen und Ausfallgarantien sowie von Sicherheiten oder für die Marktbeobachtung notwendig ist. 
+Art. 32d Abs. 2 [GZ]
+Der Bundesrat regelt für die Zwecke der Liquiditätshilfedarlehen mit Ausfallgarantie den Austausch nicht öffentlich zugänglicher Informationen zwischen dem EFD, der FINMA, der Nationalbank und ausserdem:
+a. zur Bewertung der Risiken für den eidgenössischen Haushalt: die von der FINMA und der Nationalbank an das EFD zu erteilenden Informationen; und
+b. zur Beurteilung der Liquiditätshilfe-Darlehen, der Ausfallgarantien sowie der damit zusammenhängenden finanziellen Verpflichtungen des Bundes: die vom EFD der Eidgenössischen Finanzkontrolle zu übermittelnden Unterlagen und Informationen.
+Art. 32e Titel [GZ]
+Überprüfung dieses Abschnitts
+Art. 32e Text [GZ]
+Der Bundesrat muss spätestens fünf Jahre nach Inkrafttreten der Änderung vom ... die Bestimmungen dieses Abschnitts sowie der Ausführungsbestimmungen prüfen. Er erstattet der Bundesversammlung darüber Bericht und zeigt den allfälligen Aufhebungs- oder Anpassungsbedarf auf Gesetzesstufe auf.
+Art. 34 Abs. 1 [GZ]
+... Abweichende Bestimmungen des vorliegenden Gesetzes bleiben vorbehalten.
+Art. 36 Abs. 1bis [GZ]
+Die Rangordnung der Gläubiger und die Befriedigung ihrer Forderungen innerhalb der Rangklassen nach dem Artikel 32c sind im Kollokationsplan zu berücksichtigen.
+Art. 46 Abs. 1 Bst. d [GZ]
+d. die Pflichten nach Artikel 32b verletzt.
+[VS]
+Antrag der Minderheit I [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Gemäss Mehrheit
+[VS]
+Antrag der Minderheit II [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Streichen
+[VS]
+Antrag Aeschi [GZ]
+Streichen
+Schriftliche Begründung [GZ]
+Die Botschaft zum Geschäft des Bundesrates 23.062 Bankengesetz. Änderung ("Public Liquidity Backstop") wurde am 6. September 2023 durch den Bundesrat z. H. des Parlaments verabschiedet. Der Public Liquidity Backstop (PLB) wurde im Februar 2025 einstimmig in der WAK-S sistiert. Gestützt auf Anhörungen, u. a. von zwei Rechtsprofessorinnen und zwei Ökonomen, Ständeräte hielten in der Ständeratsdebatte fest, dass die Einführung des PLB zusammen mit der gesamten Too-big-to-fail-Vorlage beraten werden sollte. Dies vor dem Hintergrund, dass zwischen den Anforderungen an die Eigenmittel und der Ausgestaltung des PLB ein enger Zusammenhang bestehe. Der Ständerat ist in der Frühjahrsession 2025 diesem Antrag gefolgt und hat beschlossen, die Beratung der Botschaft zur Einführung eines Public Liquidity Backstops (23.062) und zweier Motionen (21.3910 und 23.3462) zu sistieren. Die WAK-N hat diesem Beschluss am 1. April 2025 einstimmig zugestimmt. Eine hypothetische Einnahme in ein Entlastungspaket aufzunehmen, ohne Diskussion in den zuständigen Kommissionen, greift dem ordentlichen Gesetzgebungsverfahren vor und stellt die Budgetplanung auf eine unsichere Basis. Zudem adressiert das Entlastungspaket strukturelle Ausgabenprobleme. Die Verknüpfung mit einer noch nicht geregelten finanzmarktpolitischen Vorlage ist systemfremd und vermischt zwei getrennte Entscheidungsprozesse. Sachpolitisch ist es geboten, über den PLB als zentrales Element der Finanzstabilität zu beraten und nicht als fiskalisches Instrument. Folgende inhaltliche Gründe sprechen zusätzlich gegen die Aufnahme des PLB ins Entlastungspaket 27:
+1. Die in der Fahne zum Entlastungspaket vorgeschlagene Regelung weicht in zentralen Punkten deutlich vom PLB-Gesetzesvorschlag des Bundesrates ab. So enthält der PLB-Vorschlag gemäss Entlastungspaket bloss die Hälfte der Bestimmungen, die der Bundesrat bei der PLB-Vorlage unterbreitet hatte. Eine fundierte und seriöse Analyse der konkreten Abweichungen war sowohl für die Mitglieder der FK-N als auch für die übrigen Mitglieder des Nationalrats im gegebenen Zeitrahmen nicht möglich. Umso problematischer ist, dass die Gründe für diese erheblichen Differenzen nicht transparent dargelegt wurden. Eine solche Intransparenz erschwert eine sachgerechte parlamentarische Beurteilung und untergräbt die notwendige Nachvollziehbarkeit des Gesetzgebungsprozesses.
+2. Da die Anwendung eines PLB mit einem weitreichenden Konkursprivileg verbunden ist, kein Anspruch besteht und im Falle eines Einsatzes des PLB bereits substanzielle Zinsen und Prämien an den Bund zu zahlen wären, fehlt einer zusätzlichen Abgeltungspauschale eine sachlich nachvollziehbare Begründung. Eine im Voraus zu entrichtende Abgeltung (ex-ante) steht im Widerspruch zur Tatsache, dass es für eine Bank keinen rechtlichen Anspruch auf einen PLB gibt. Zu diesem Schluss ist auch der Bundesrat in seiner Vernehmlassung zur Einführung eines PLB vom Mai 2023 gekommen, indem er eine ex-ante-Abgeltung als "nicht begründbar" verworfen hatte.
+[VS]
+Proposition de la majorité [GZ]
+Art. 10b titre [GZ]
+Collaboration du DFF, de la FINMA et de la Banque nationale en vue de prévenir ou de maîtriser la défaillance d'une banque d'importance systémique
+Art. 10b texte [GZ]
+Si la FINMA estime, notamment après avoir évalué les risques encourus par une banque d'importance systémique, qu'il pourrait être nécessaire d'ordonner une des mesures visées à l'article 25 alinéa 1, la FINMA communique immédiatement son évaluation au DFF et à la Banque nationale. Une fois avisée par la FINMA, la Banque nationale communique son évaluation au DFF, notamment en ce qui concerne les risques pour l'économie et le système financier suisses.
+Art. 30b al. 3 let. a[GZ]
+a. es créances privilégiées de première et de deuxième classe au sens de l'article 219 alinéa 4 LP et les créances visées à l'article 32c alinéa 1, dans la limite des privilèges accordés ;
+Chapitre XIa titre[GZ]
+Octroi par la Confédération de garanties du risque de défaillance pour les prêts d'aide sous forme de liquidités de la Banque nationale à des banques d'importance systémique
+Art. 32a titre [GZ]
+Garanties du risque de défaillance
+Art. 32a al. 1 [GZ]
+La Confédération peut octroyer à la Banque nationale des garanties du risque de défaillance subsidiaires pour les prêts d'aide sous forme de liquidités qui ont été accordés à des banques d'importance systémique ou faisant partie d'un groupe financier d'importance systémique, si
+a. la procédure d'assainissement de l'emprunteur a été engagée ou est sur le point de l'être; et
+b. sans l'octroi de tels prêts, l'économie et le système financier suisses risquent de subir des dommages considérables.
+Art. 32a al. 2 [GZ]
+Une fois par année, la Confédération prélève auprès des banques qui sont d'importance systémique ou font partie d'un groupe financier d'importance systémique un forfait pour risque lié à une éventuelle mise à disposition d'une garantie du risque de défaillance. Le forfait équivaut au produit d'un taux de calcul unique et d'une base de calcul déterminée pour chacune des banques.
+Art. 32a al. 3 [GZ]
+La Confédération peut prétendre à une prime pour la mise à disposition d'une garantie du risque de défaillance. La prime de mise à disposition dépend du montant de la garantie.
+Art. 32a al. 4 [GZ]
+La Confédération et la Banque nationale peuvent chacune prétendre à une prime de risque au titre de compensation des risques qu'elles courent du fait de l'octroi d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance. Les primes de risque dépendent du montant versé au titre d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance.
+Art. 32a al. 5 [GZ]
+La Banque nationale peut prétendre à des intérêts sur les prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance.
+Art. 32a al. 6 [GZ]
+Les frais pour des prestations de tiers liés aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance de la Confédération, de la Banque nationale ou de la FINMA sont mis à la charge de l'emprunteur.
+Art. 32a al. 7 [GZ]
+Le Conseil fédéral règle notamment :
+a. les mesures que l'emprunteur doit avoir épuisées pour trouver des sources de financement ou obtenir des garanties ;
+b. le taux et la base de calcul du forfait ainsi que le calcul et la perception de la prime de mise à disposition, des primes de risque et des intérêts ;
+c. le moment et l'étendue du droit de la Banque nationale à la prise en charge d'une perte définitive résultant des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ainsi que les conditions dans lesquelles ce droit devient exigible ;
+d. les autres conditions requises pour bénéficier d'un prêt d'aide sous forme de liquidités assorti d'une garantie du risque de défaillance, notamment les confirmations nécessaires de la FINMA et de la Banque nationale ;
+e. les obligations de la FINMA et de la Banque nationale en matière de réduction des risques, de surveillance et de rapports.
+Art. 32b titre [GZ]
+Obligations de l'emprunteur liées aux prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance
+Art. 32b al. 1 [GZ]
+L'emprunteur et les filiales qui y sont directement ou indirectement liées ne sont pas autorisés à exécuter les opérations suivantes :
+a. avaliser et verser des dividendes et des tantièmes à des personnes appartenant ou non au groupe de l'emprunteur ;
+b. restituer des fonds propres de base durs, des fonds propres de base supplémentaires, des fonds propres complémentaires et des fonds supplémentaires destinés à absorber les pertes ;
+c. octroyer et rembourser des prêts aux propriétaires de la société mère du groupe ;
+Art. 32b al. 2 [GZ]
+L'emprunteur et les sociétés du groupe qui y sont directement ou indirectement liées n'effectuent pas d'acte qui pourrait retarder ou compromettre le remboursement des prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance ou le paiement de la totalité des primes et des intérêts visés à l'article 32a, ni n'omettent d'acte qui favoriserait le remboursement des prêts ainsi que le paiement de la totalité de ces primes et intérêts
+Art. 32b al. 3 [GZ]
+L'emprunteur est tenu de rembourser les prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance avant les autres prêts d'aide sous forme de liquidités que la Banque nationale lui a octroyés.
+Art. 32b al. 4 [GZ]
+Le Conseil fédéral règle les obligations de l'emprunteur, y compris les exceptions:
+a. des obligations de l'emprunteur visées aux alinéas 1 et 2, en particulier :
+1. pour les obligations ordinaires préexistantes de payer des intérêts ou des charges d'amortissement en lien avec les opérations visées à l'alinéa 1 lettres b ou c; et
+2. lorsque l'emprunteur ou le groupe financier est acquis par une société tierce et qu'il est absorbé par une unité de cette même société tierce.
+b. de l'obligation de rembourser en priorité les prêts d'aide sous forme de liquidités assortis d'une garantie de défaillance.
+Art. 32c titre [GZ]
+Privilège des créances découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance
+Art. 32c al. 1 [GZ]
+Les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus sont attribués à la troisième classe au sens de l'article 219 alinéa 4 LP.
+Art. 32c al. 2 [GZ]
+S'il y en a, les créances de la troisième classe sont, en dérogation à l'article 220 alinéa 1 LP, honorées dans l'ordre suivant :
+a. les créances découlant de comptes de libre passage sous forme d'épargne pure prévus par le Conseil fédéral sur la base de l'article 26 alinéa 1 de la loi du 17 décembre 1993 sur le libre passage et les créances découlant de dépôts d'épargne sur des comptes de la prévoyance individuelle liée visée à l'article 82 alinéa 1 lettre b de la loi du 25 juin 1982 sur la prévoyance professionnelle vieillesse, survivants et invalidité ;
+b. les créances de la Banque nationale découlant de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, les primes courues dues à la Banque nationale et à la Confédération et les intérêts courus ;
+c. toutes les autres créances de la troisième classe.
+Art. 32d titre [GZ]
+Traitement des données et échange d'informations
+Art. 32d al. 1 [GZ]
+Le DFF, la FINMA, la Banque nationale, le CDF et les tiers chargés de l'exécution des dispositions du présent chapitre peuvent traiter et se communiquer mutuellement des données personnelles et des données concernant des personnes morales, y compris des données sensibles au sens de l'article 5 lettre c chiffres 1, 2, 5 et 6, de la loi du 25 septembre 2020 sur la protection des données et des données sensibles concernant des personnes morales au sens de l'article 57r alinéa 2 de la loi du 21 mars 1997 sur l'organisation du gouvernement et de l'administration, ainsi que d'autres informations, dans la mesure où cela est nécessaire à l'exécution des dispositions du présent chapitre, notamment pour l'octroi, l'administration, la surveillance, le contrôle et le traitement des prêts d'aide sous forme de liquidités et des garanties du risque de défaillance ainsi que des sûretés, ou pour l'observation du marché.
+Art. 32d al. 2 [GZ]
+Le Conseil fédéral règle, dans le cadre de prêts d'aide sous forme de liquidités assortis d'une garantie du risque de défaillance, l'échange d'informations non accessibles au public entre le DFF, la FINMA, la Banque nationale et, en outre :
+a. pour l'évaluation des risques pour le budget de la Confédération : les informations par que la FINMA et la Banque nationale doivent fournir au DFF ; et
+b. pour l'évaluation des prêts d'aide sous forme de liquidités, des garanties du risque de défaillance ainsi que des engagements financiers de la Confédération qui y sont liés : les documents et informations que le DFF doit transmettre au Contrôle fédéral des finances.
+Art. 32e titre [GZ]
+Examen des dispositions du présent chapitre
+Art. 32e texte [GZ]
+Cinq ans au plus tard après l'entrée en vigueur de la modification du ..., le Conseil fédéral réexamine les dispositions du présent chapitre ainsi que les dispositions d'exécution. Il fait rapport à l'Assemblée fédérale et détermine les dispositions législatives qu'il y a lieu éventuellement de modifier ou d'abroger.
+Art. 34 al. 1 [GZ]
+... Les dispositions dérogatoires de la présente loi sont réservées.
+Art. 36 al. 1bis [GZ]
+L'ordre des créanciers et le paiement de leurs créances selon l'ordre visé à l'article 32c sont pris en compte dans l'état de collocation.
+Art. 46 al. 1 let d[GZ]
+d. contrevient aux obligations prévues à l'article 32b.
+[VS]
+Proposition de la minorité I [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Selon majorité
+[VS]
+Proposition de la minorité II [GZ]
+(Funiciello, Fehlmann Rielle, Gysi Barbara, Wyss, Zybach)[GZ]
+Biffer
+[VS]
+Proposition Aeschi [GZ]
+Biffer
+[VS]
+Le président (Page Pierre-André, président): La majorité et la minorité I proposent différentes modifications du plan financier. Les votes valent également pour l'arrêté fédéral IIa concernant les mesures d'allègement du budget 2027 arrêtées dans le plan financier pour les années 2027-2029.
 </t>
   </si>
 </sst>
@@ -180,8 +382,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I5" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I6" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I6"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -624,6 +826,35 @@
         <v>36</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-05
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -172,7 +172,7 @@
 Der Bund erhebt von den Banken, die systemrelevant oder Teil einer systemrelevanten Finanzgruppe sind, jährlich eine Pauschale für das Risiko einer allfälligen Bereitstellung einer Ausfallgarantie. Die Pauschale entspricht dem Produkt aus einem einheitlichen Bemessungssatz und einer für jede Bank berechneten Bemessungsgrundlage. 
 Art. 32a Abs. 3 [GZ]
 Der Bund hat Anspruch auf eine Prämie für die Bereitstellung einer Ausfallgarantie. Die Bereitstellungsprämie bemisst sich nach der Höhe der Ausfallgarantie. 
-32a Abs. 4 [GZ]
+Art. 32a Abs. 4 [GZ]
 Der Bund und die Nationalbank haben Anspruch auf je eine Risikoprämie zur Abgeltung der mit einem Liquiditätshilfe-Darlehen mit Ausfallgarantie übernommenen Risiken. Die Risikoprämien bemessen sich nach der Höhe der ausbezahlten Liquiditätshilfe-Darlehen mit Ausfallgarantie. 
 Art. 32a Abs. 5 [GZ]
 Die Nationalbank hat Anspruch auf Zinsen auf Liquiditätshilfe-Darlehen mit Ausfallgarantie.
@@ -361,6 +361,31 @@
 Abschliessend kann ich sagen, dass die SVP-Fraktion im Block 4 dem Entwurf des Bundesrates folgt und die Minderheitsanträge, die in eine andere Richtung gehen, ablehnt.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">370058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Andrey Gerhard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds der AHV, IV und EO, sodass keine Belastung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ich möchte im Namen der Kommission über die Botschaft des Bundesrates vom 12. September vergangenen Jahres zu einem Verpflichtungskredit von 66,1 Millionen Franken für die digitale Transformation der zentralen Ausgleichsstelle in den Jahren 2026 bis 2032 berichten. Die Gesamtkosten des Programms belaufen sich auf 123,3 Millionen Franken, wovon gut die Hälfte durch interne Ressourcen der ZAS gedeckt wird. Die Finanzierung erfolgt über die Ausgleichsfonds der AHV, IV und EO, sodass keine Belastung des Bundeshaushaltes entsteht. 
+Ziel des Vorhabens ist die umfassende Modernisierung der Organisation, der Geschäftsprozesse und der Informatiksysteme der ZAS, die als operatives Rückgrat der ersten Säule zentrale Register führt, die Finanzflüsse steuert und weltweit über eine Million Renten auszahlt. Die bestehenden Systeme seien technisch überaltert und stark fragmentiert, was die Automatisierung hemme, die Anpassung an gesetzliche Änderungen verteuere und die Datensicherheit gefährde. Ohne eine tiefgreifende Transformation wäre die ZAS laut eigenen Aussagen künftig nicht mehr in der Lage, Qualität und Effizienz ihrer Leistungen sicherzustellen. 
+Das Programm ist ein Schlüsselprojekt der Bundesverwaltung und als solches eingestuft. Es umfasst rund zehn miteinander verknüpfte Projekte, die in drei Phasen bis ins Jahr 2032 laufen. Kernpunkte sind die Umgestaltung der Prozesse hin zu vier bereichsübergreifenden Querschnittsprozessen, die Migration auf die standardisierte IT-Architektur, die Integration marktgängiger Lösungen und die Einführung eines neuen Betriebsmodells. Damit sollen die Silostrukturen aufgebrochen, die Automatisierung vorangetrieben und die Interoperabilität mit anderen Projekten der ersten Säule gewährleistet werden.
+Die Transformation soll es ermöglichen, das wachsende Arbeitsvolumen ohne zusätzliche Stellen zu bewältigen. Das Einsparpotenzial wird auf bis zu 80 Vollzeitäquivalente über zehn Jahre geschätzt, wobei die tatsächliche Wirkung vom Automatisierungsgrad und der Stabilität der Prozesse abhängen wird. Neben Effizienzgewinnen werden kürzere Bearbeitungszeiten, eine höhere Datensicherheit und eine bessere Anpassungsfähigkeit an gesetzliche Änderungen erwartet. 
+Ihre Finanzkommission hat die Vorlage eingehend beraten. In der Eintretensdebatte wurde die strategische Bedeutung des Projekts unumstritten anerkannt. Angesichts der demografischen Entwicklung, der steigenden Mobilität und der veralteten Infrastruktur wurde die Notwendigkeit einer Modernisierung von allen Seiten bestätigt. Diskutiert wurden Fragen zur Kontrolle der Effizienzgewinne, zu Teuerungsannahmen sowie zur Vermeidung von Anbieterabhängigkeit. Die Kommission begrüsst die geplante Standardisierung und die Reuse-Strategie, um bestehende Lösungen innerhalb der Bundesverwaltung zu nutzen. Auch die Governance-Struktur mit der Einbindung der Bundeskanzlei und der Begleitung durch die Eidgenössische Finanzkontrolle wurde positiv bewertet. 
+Die Kommission hat sich über die Konsequenzen des neuen Bundesgesetz über den Einsatz elektronischer Mittel zur Erfüllung von Behördenaufgaben (EMBAG) informiert, das die Veröffentlichung des Quellcodes solcher behördlicher Software verlangt. Der Kommission wurde versichert, dass es diesbezüglich keine Probleme gebe, weil die Rechte der bestehenden Software weitgehend beim Bund liegen und sich das mit dem neuen Programm nicht ändern werde. 
+Ihre Finanzkommission sieht im Programm eine notwendige Investition in die Zukunftsfähigkeit der ersten Säule und empfiehlt dem Rat einstimmig, auf die Vorlage einzutreten und den Verpflichtungskredit zu bewilligen.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -407,8 +432,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I7" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I8" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I8"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -909,6 +934,35 @@
         <v>45</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" t="s">
+        <v>50</v>
+      </c>
+      <c r="I8" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-09
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -89,10 +89,10 @@
     <t xml:space="preserve">DE</t>
   </si>
   <si>
-    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vor, dass dieses doch komplexe Thema in der zuständigen Kommission vertieft behandelt wird, damit der Rat dann auf einer gesicherten Grundlage den richtigen Entscheid treffen kann.
+    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle (EFK) darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ih</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle (EFK) darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vor, dass dieses doch komplexe Thema in der zuständigen Kommission vertieft behandelt wird, damit der Rat dann auf einer gesicherten Grundlage den richtigen Entscheid treffen kann.
 Mein Antrag lautet also: Überweisung an die zuständige Kommission.
 </t>
   </si>
@@ -112,7 +112,8 @@
     <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzresso</t>
   </si>
   <si>
-    <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik. Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
+    <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik.
+Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
 </t>
   </si>
   <si>

</xml_diff>

<commit_message>
Update debates data - 2026-03-10
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -403,6 +403,29 @@
     <t xml:space="preserve">Monsieur le conseiller national Amoos, Sipacfutur est un projet clé de la Confédération. À ce titre, il a été accompagné par le Contrôle fédéral des finances, qui a publié six rapports à son propos. Les recommandations des cinq premiers rapports ont été mises en oeuvre, ce qui a été attesté dans le sixième et dernier rapport. Ce dernier attirait encore l'attention sur la phase de migration entre l'ancien et le nouveau système. La migration a donc fait l'objet d'une attention particulière et a été effectuée sans problèmes notables. Des dysfonctionnements importants sont apparus par la suite et ont causé du retard dans certains paiements, ce qui est regrettable. Depuis février, le système est nettement plus stable. Actuellement, on travaille à la résorption du retard et à l'amélioration de la performance du système - voir aussi les questions 26.7131 et 26.7133 Mahaim.
 </t>
   </si>
+  <si>
+    <t xml:space="preserve">370837</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20260310</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dans cette affaire, je ne peux que répéter une nouvelle fois mon plaidoyer en faveur d'une action efficace et rapide. Aux yeux du Conseil fédéral, un accord reste la façon la plus simple et la plus directe d'y parvenir. Lancer maintenant un processus législatif nous ferait perdre un temps précieux, d'autant plus que la consultation publique a montré que la majorité des participants approuvent l'accord et la démarche du Conseil fédéral. Je reviendrai plus tard sur les résultats de la consultation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dans cette affaire, je ne peux que répéter une nouvelle fois mon plaidoyer en faveur d'une action efficace et rapide. Aux yeux du Conseil fédéral, un accord reste la façon la plus simple et la plus directe d'y parvenir. Lancer maintenant un processus législatif nous ferait perdre un temps précieux, d'autant plus que la consultation publique a montré que la majorité des participants approuvent l'accord et la démarche du Conseil fédéral. Je reviendrai plus tard sur les résultats de la consultation.
+Le Conseil fédéral est certain d'avoir choisi la bonne voie. Lors de la visite de la première ministre Ioulia Sviridenko en Suisse fin août, elle a explicitement souligné l'efficacité des instruments suisses pour inclure le secteur privé. Elle considère l'approche suisse comme un modèle pour d'autres pays. L'Ukraine elle-même recherche, en complément des instruments classiques de la coopération internationale, des investissements privés afin de stabiliser son économie. Le Conseil fédéral prend ce besoin très au sérieux et a fait de l'implication de l'économie privée suisse dans la reconstruction de l'Ukraine une priorité en allouant un montant de 500 millions de francs pour les quatre prochaines années. Le fait que nous ne pouvons simplement pas attendre est particulièrement évident au vu des derniers développements en Ukraine. Compte tenu de la grave crise énergétique sur place et à la suite d'une demande du gouvernement ukrainien, le Conseil fédéral a décidé le 11 février dernier d'adopter un plan d'aide humanitaire pour la livraison de produits énergétiques de première nécessité avec un plafond de 32 millions de francs. Ce plan d'aide va permettre d'acquérir, de livrer et d'installer 18 modules électriques fonctionnant au gaz naturel et jusqu'à 80 générateurs diesel de différentes puissances des fournisseurs suisses.
+Depuis le dépôt de la motion, quels sont les derniers développements ? Cette motion de la Commission de politique extérieure du Conseil des États a été acceptée par ce dernier, par 33 voix contre 12. C'était le 19 mars de l'année passée. Vous, le Conseil national, en revanche, avez rejeté le 20 mars 2025, par 105 voix contre 74 et 12 abstentions, une motion de votre Commission de politique extérieure dont le contenu était exactement le même. Je vous demande de rester cohérents et d'en rester à votre position. Parallèlement, lors de la consultation du mandat de négociation pour un traité international avec l'Ukraine, les Commissions de politique extérieure des deux conseils ont accepté ce mandat. C'était en février et en avril dernier. Ainsi, elles ont accepté la démarche du Conseil fédéral concernant la base légale pour l'aide à l'Ukraine. Cela nous a permis de faire avancer les travaux pour la négociation d'un traité avec l'Ukraine. Les négociations entre la Suisse et l'Ukraine se sont déroulées de manière très constructive et le résultat des négociations correspond aux objectifs de la Suisse. Tous ces échanges nous ont permis d'établir une relation de confiance entre notre pays et l'Ukraine. La collaboration est étroite. Nous devons bâtir sur cette confiance. Si la motion devait être adoptée, ce travail se poursuivrait, mais cela marquerait tout de même un sérieux coup dans nos relations avec l'Ukraine et cela freinerait ce mouvement positif que nous connaissons actuellement.
+Concernant les prochaines étapes pour l'approbation de l'accord par l'Assemblée fédérale, le Conseil fédéral a soumis vendredi dernier, le 6 mars, son message au Parlement pour l'approbation du traité. Le traité fera également l'objet de la possibilité d'un référendum.
+J'en viens maintenant, comme je vous l'ai dit tout à l'heure, à une brève appréciation des résultats de la consultation publique concernant le traité. Celle-ci s'est terminée le 12 novembre dernier et nous avons reçu un total de 53 prises de position dont 24 cantons, 4 partis politiques, 5 associations faîtières de l'économie et 20 ONG. Je peux vous informer, et je suis heureux de pouvoir vous dire qu'une majorité des participants se sont exprimés en faveur de l'accord que le Conseil fédéral a signé. Les principales raisons qui motivent l'approbation de l'accord sont les suivantes.
+Les principales raisons qui motivent l'approbation de l'accord sont les suivantes. L'importance du soutien à l'Ukraine pour la stabilité en Europe et, par conséquent, l'engagement de la Suisse, sont reconnus. L'implication du secteur privé suisse est considérée comme indispensable pour la reconstruction en Ukraine. L'accord permet d'apporter une aide rapide à l'Ukraine. L'approche de partenariat dans le cadre de laquelle l'Ukraine et la Suisse collaborent étroitement pour choisir les projets est saluée. La protection juridique des moyens engagés par le biais du monitorage, de l'évaluation, du contrôle par le Contrôle fédéral des finances ainsi que par le respect des principes de l'état de droit et de la démocratie, des droits de l'homme et de la lutte contre la corruption ont été soulignés positivement.
+Le Conseil fédéral reste convaincu que l'accord négocié avec l'Ukraine représente une solution élégante et efficiente qui nous permet de résoudre les questions juridiques relatives aux aides financières prévues ainsi que de régler les obligations des deux parties. Alors que les arguments en faveur du traité international restent les mêmes, nous sommes aujourd'hui plus avancés et avons la preuve que notre approche rencontre un écho positif en Ukraine et en Suisse. Au moment de la clôture du premier appel d'offres, près de 80 propositions avaient été reçues, venant de 60 entreprises suisses. Douze projets ont été sélectionnés, et leur mise en oeuvre est en bonne route. Les projets couvrent des thèmes tels que l'approvisionnement énergétique, l'hébergement pour les personnes déplacées à l'intérieur du pays ou les chemins de fer. Le budget total des projets sélectionnés s'élève à plus de 112 millions de francs, dont 93 millions sont financés par la Suisse, le reste étant pris en charge par les entreprises et par leurs partenaires ukrainiens.
+Il convient également de mentionner la participation des ONG suisses dans le cadre de ces projets. Elles apportent en effet leur expertise au secteur privé, une piste qui pourrait être approfondie pour de futurs appels à propositions. Entre-temps, nous avons lancé un deuxième appel à propositions le 9 janvier et le délai pour soumettre les projets échoit cette semaine. Compte tenu des retours positifs du marché, nous attendons à nouveau un grand nombre de propositions de projets.
+En conclusion, je suis persuadé que nous, Parlement et Conseil fédéral, avons le même objectif : fournir une aide à l'Ukraine le plus vite possible, là où elle est nécessaire, en encourageant les entreprises suisses à livrer des biens et des services urgents pour sa reconstruction, dont l'Ukraine ne dispose pas actuellement. Nous pouvons ainsi créer un levier ou un effet de levier pour relancer l'économie ukrainienne. Grâce à l'accord que nous avons négocié et signé, nous pourrons atteindre cet objectif dès l'automne prochain. Je vous invite à continuer sur cette voie, qui est efficace et à ne pas en ouvrir une deuxième qui pourrait ralentir le processus de soutien et utiliserait des ressources aujourd'hui utiles à la mise en oeuvre du programme suisse pour l'Ukraine.
+Je vous invite dès lors à accepter la démarche que nous suivons et à rejeter une deuxième fois cette motion qui a, je le répète, les mêmes termes que la première motion.
+Si vous deviez l'accepter, le Conseil fédéral poursuivrait le processus de ratification de l'accord. Il élaborera en parallèle une loi, et nous pourrons ainsi faire de notre mieux pour que le soutien à l'Ukraine et les secteurs privés en Suisse puissent débuter l'année prochaine. Je le répète : il serait administrativement et politiquement extrêmement dommage que vous suiviez cet aspect. Je vous invite vivement à rejeter cette motion, pour des raisons d'efficacité.
+</t>
+  </si>
 </sst>
 </file>
 
@@ -449,8 +472,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I9" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="A1:I9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I10" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="A1:I10"/>
   <tableColumns count="9">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="MeetingDate"/>
@@ -1007,6 +1030,33 @@
         <v>56</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10"/>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s">
+        <v>59</v>
+      </c>
+      <c r="I10" t="s">
+        <v>60</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>

</xml_diff>

<commit_message>
Update debates data - 2026-03-13
</commit_message>
<xml_diff>
--- a/Debats_CDF_EFK.xlsx
+++ b/Debats_CDF_EFK.xlsx
@@ -93,7 +93,7 @@
   </si>
   <si>
     <t xml:space="preserve">Dieses Thema ist von grosser forschungs- und wirtschaftspolitischer Bedeutung. Es ist komplex und wichtig. In mehreren Berichten hat die Eidgenössische Finanzkontrolle (EFK) darauf hingewiesen, dass in diesem Bereich die rechtlichen Grundlagen zu verbessern seien, um die Mehrfachnutzung öffentlicher Daten sicherzustellen, insbesondere auch durch Aktivitäten des Bundesamtes für Statistik. Die Ablehnung des Vorstosses durch den Bundesrat kommt in dieser Situation etwas überraschend. Ich schlage Ihnen vor, dass dieses doch komplexe Thema in der zuständigen Kommission vertieft behandelt wird, damit der Rat dann auf einer gesicherten Grundlage den richtigen Entscheid treffen kann.
-Mein Antrag lautet also: Überweisung an die zuständige Kommission.
+Mein Antrag lautet also: Zuweisung an die zuständige Kommission.
 </t>
   </si>
   <si>
@@ -113,7 +113,7 @@
   </si>
   <si>
     <t xml:space="preserve">Ich habe den Satz des Bundesrates gelesen: "Ohne verbindliche Standards und einheitliche Beschreibung der Daten aus vertrauenswürdigen Quellen können KI-gestützte Analysen weder verlässlich noch effizient durchgeführt werden." Da sind wir uns einig. Dann kommt aber die Kehrtwendung. Wir sind uns nicht einig, ob die Instrumente, die dem Bundesrat oder der Verwaltung heute zur Verfügung stehen, ausreichen, um das Ziel zu erreichen. Ich glaube, die Hindernisse sind eben mehr als nur die Finanzressourcen, wie der Bundesrat suggeriert, sondern es bestehen, wie Herr Kollege Stark angetönt hat, auch Regelungslücken. Ich gebe der Kommission wirklich mit auf den Weg, dass sie die EFK-Berichte genau anschaut, in denen es heisst, es fehle an Weisungskompetenzen und an Durchsetzungskraft etwa des Bundesamtes für Statistik.
-Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Überweisung an die Kommission.
+Ich glaube, hier ist schon etwas mehr zu tun. Aber um Klärung zu erhalten, bin ich einverstanden mit dem Antrag zur Zuweisung an die Kommission.
 </t>
   </si>
   <si>

</xml_diff>